<commit_message>
add Essentials of Team Collaboration to Essential Lessons for First-Time Managers.xlsx
</commit_message>
<xml_diff>
--- a/Essential Lessons for First-Time Managers.xlsx
+++ b/Essential Lessons for First-Time Managers.xlsx
@@ -5,16 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.go\Videos\Essential Lessons for First-Time Managers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Career\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF7CF7D-A690-421F-A93F-6AF5DA8F2976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EF21AC-276C-4833-B9B5-E6FB67EDCD82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A70EA376-3E6C-4188-8422-C32BD3C80C75}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A70EA376-3E6C-4188-8422-C32BD3C80C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Essentials of Team Collaboratio" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Essentials of Team Collaboratio'!$A$2:$G$59</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="208">
   <si>
     <t>Congratulations on being a manager(Viewed)</t>
   </si>
@@ -336,19 +340,435 @@
   </si>
   <si>
     <t>4. The People Stuff: Leadership (4. Authenticity, transparency, and vulnerability)</t>
+  </si>
+  <si>
+    <t>Welcome to Essentials of Team Collaboration</t>
+  </si>
+  <si>
+    <t>1m 38s</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Why team collaboration is necessary</t>
+  </si>
+  <si>
+    <t>3m 27s</t>
+  </si>
+  <si>
+    <t>1. Setting the Stage for Strong Team Collaboration</t>
+  </si>
+  <si>
+    <t>Six key questions for effective collaboration</t>
+  </si>
+  <si>
+    <t>2m 51s</t>
+  </si>
+  <si>
+    <t>Identify the right team composition</t>
+  </si>
+  <si>
+    <t>2m 22s</t>
+  </si>
+  <si>
+    <t>Clarify the team's goal and purpose</t>
+  </si>
+  <si>
+    <t>2m 37s</t>
+  </si>
+  <si>
+    <t>Clarify constraints, expectations, and processes up front</t>
+  </si>
+  <si>
+    <t>2m 24s</t>
+  </si>
+  <si>
+    <t>2. Five Tactics to Encourage Healthy Team Collaboration</t>
+  </si>
+  <si>
+    <t>Develop team ground rules</t>
+  </si>
+  <si>
+    <t>2m 16s</t>
+  </si>
+  <si>
+    <t>Build relationships early and often(Viewed)</t>
+  </si>
+  <si>
+    <t>3m 7s</t>
+  </si>
+  <si>
+    <t>Identify team members' preferred communication mode</t>
+  </si>
+  <si>
+    <t>2m 39s</t>
+  </si>
+  <si>
+    <t>Tips for great online collaboration</t>
+  </si>
+  <si>
+    <t>2m 56s</t>
+  </si>
+  <si>
+    <t>Take periodic temperature checks</t>
+  </si>
+  <si>
+    <t>2m 23s</t>
+  </si>
+  <si>
+    <t>6 questions</t>
+  </si>
+  <si>
+    <t>Conclusion</t>
+  </si>
+  <si>
+    <t>Develop best practices to enhance team collaboration</t>
+  </si>
+  <si>
+    <t>Team collaboration challenge</t>
+  </si>
+  <si>
+    <t>1m 31s</t>
+  </si>
+  <si>
+    <t>2 questions</t>
+  </si>
+  <si>
+    <t>Take exam</t>
+  </si>
+  <si>
+    <t>Essentials of Team Collaboration</t>
+  </si>
+  <si>
+    <t>Why should you analyze team composition early in the process?</t>
+  </si>
+  <si>
+    <t>to identify potential resource needs and issues so they can be promptly mitigated or addressed
+Early consideration of resources needs and issues provides an opportunity to proactively address potential problems down the road.</t>
+  </si>
+  <si>
+    <t>You want to determine whether or not your team has a shared vision for completing a project. What makes clarifying the "why" important, in terms of why the project is being done?</t>
+  </si>
+  <si>
+    <t>Ellie is leading a new project team. What is a critical question the team should address during their work on constraints, expectations, and processes?</t>
+  </si>
+  <si>
+    <t>"How will we work together?"
+Ellie should make sure the team agrees on the "how," which will confirm whether they have developed efficient and effective processes.</t>
+  </si>
+  <si>
+    <t>What is the overarching purpose of the 6 key questions for effective collaboration?</t>
+  </si>
+  <si>
+    <t>to clarify and define team parameters and expectations
+Asking these six questions (particularly at the beginning of a team experience) provides an opportunity to discuss, clarify, and define.</t>
+  </si>
+  <si>
+    <t>to help motivate and inspire the team to work on the project
+Clarifying the "why," or the mission, makes people care about the project's goals and tasks while helping to motivate them as well.</t>
+  </si>
+  <si>
+    <t>You are meeting with your team to set ground rules on a new collaborative project. How can you best start in determining which ground rules to have?</t>
+  </si>
+  <si>
+    <t>Ask each team member to present a ground rule from a previous project that worked effectively.
+Since the ground rules reflect the various personalities in the group, the team members will more easily accept and support them.</t>
+  </si>
+  <si>
+    <t>You're preparing for a meeting with your new team. What might be an easy and effective way to encourage relationship building?</t>
+  </si>
+  <si>
+    <t>Ask team members to work in pairs of two or three on key tasks, instead of assigning tasks to individual owners.
+Activities that encourage team members to connect with each other provides opportunities for relationship building. This might include traditional icebreaker/getting to know you type activities, being paired together to work on social activities, etc.</t>
+  </si>
+  <si>
+    <t>You acknowledge the importance of discussing individual communications preferences with your new team. What might be a key question to ask and discuss?</t>
+  </si>
+  <si>
+    <t>Which is the most effective principle for teams to adopt when considering online collaboration?</t>
+  </si>
+  <si>
+    <t>Identify user-friendly tools featuring functionality that increases the team's efficiency and effectiveness.
+Online collaboration tools can be helpful, but it's important for the team to focus less on a specific application and more so on the functionality that will make the team more effective and efficient.</t>
+  </si>
+  <si>
+    <t>Why is it important for a team to take a "temperature check" when working on a project?</t>
+  </si>
+  <si>
+    <t>to identify what is working and what is not working
+A "temperature check" helps the team identify potential changes or enhancements that can be made to help the project run more efficiently and effectively.</t>
+  </si>
+  <si>
+    <t>What is the central purpose of conducting periodic debrief sessions?</t>
+  </si>
+  <si>
+    <t>They determine what is working well and what could be improved from the team's perspective.
+Debriefing is a powerful tool that highlights improvement opportunities and reinforces what is working well. Debrief output provides the team a roadmap for how the group may want to make adjustments to improve going forward.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">What are some of your communication pet peeves?
+Correct
+This question elicits the type of information you're seeking about individual communication preferences. This line of inquiry provides tangible insight about how to best communicate with each team member.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Debriefing is a powerful tool that highlights improvement opportunities and reinforces what is working well. Debrief output provides the team a roadmap for how the group may want to make adjustments to improve going forward.</t>
+    </r>
+  </si>
+  <si>
+    <t>What is a best practice Marcus can use to foster collaboration on his team?</t>
+  </si>
+  <si>
+    <t>Discuss communication preferences with the team.
+Communication is essential to collaboration, so it is important for Marcus to understand his team members' preferences.</t>
+  </si>
+  <si>
+    <t>What can Sylvie do to help determine where there might be potential cracks in her team's foundation?</t>
+  </si>
+  <si>
+    <t>Review the who, what, why, where, when, and how questions.
+Sylvie can use these six questions to review, clarify, and define team parameters and then determine where they need to make adjustments.</t>
+  </si>
+  <si>
+    <t>If you want your team to be truly collaborative, which approach should you use?</t>
+  </si>
+  <si>
+    <t>Select an answer:</t>
+  </si>
+  <si>
+    <t>Determine a consistent communication mode for your team.</t>
+  </si>
+  <si>
+    <t>Rotate the leader for team meetings.</t>
+  </si>
+  <si>
+    <t>Continually check in with the team to identify what is working and what is not working.</t>
+  </si>
+  <si>
+    <t>Assume all your team members have the same work style.</t>
+  </si>
+  <si>
+    <t>What is the core purpose of team ground rules?</t>
+  </si>
+  <si>
+    <t>Leaders can define expectations for team members to effectively follow.</t>
+  </si>
+  <si>
+    <t>The team can establish mutual expectations around how they want to work together.</t>
+  </si>
+  <si>
+    <t>Each person can define preferences for how they want to work.</t>
+  </si>
+  <si>
+    <t>Management can clarify what stellar performance looks like</t>
+  </si>
+  <si>
+    <t>You realize the importance of relationship building for your newly organized team. What is the most important thing to consider as you encourage new relationships and connections?</t>
+  </si>
+  <si>
+    <t>The cost of a one-day retreat is worth it for the relationships it will build.</t>
+  </si>
+  <si>
+    <t>Building relationships is incremental and takes time.</t>
+  </si>
+  <si>
+    <t>Relationships within the team are more important than relationships across teams.</t>
+  </si>
+  <si>
+    <t>Team members should be left to build their relationships organically.</t>
+  </si>
+  <si>
+    <t>The primary benefit of a debrief is to _____.</t>
+  </si>
+  <si>
+    <t>figure out what is working well and what should potentially be changed moving forward as it relates to the team dynamics or overall project progress.</t>
+  </si>
+  <si>
+    <t>pause the team's work</t>
+  </si>
+  <si>
+    <t>energize the team for the next project</t>
+  </si>
+  <si>
+    <t>highlight the accomplishments of the team</t>
+  </si>
+  <si>
+    <t>What is a major difficulty in finding a single online tool for virtual collaboration?</t>
+  </si>
+  <si>
+    <t>There is a limited number of tools available to choose from.</t>
+  </si>
+  <si>
+    <t>Collaboration tools are too expensive.</t>
+  </si>
+  <si>
+    <t>There are team members who do not have access to online collaboration tools.</t>
+  </si>
+  <si>
+    <t>There are so many tools available to choose from.</t>
+  </si>
+  <si>
+    <t>What is a key risk of if you don't clearly define a team's purpose and goals?</t>
+  </si>
+  <si>
+    <t>a less efficient and effective team</t>
+  </si>
+  <si>
+    <t>poor deliverable quality</t>
+  </si>
+  <si>
+    <t>overspending the team budget</t>
+  </si>
+  <si>
+    <t>low team morale</t>
+  </si>
+  <si>
+    <t>What should be discussed and agreed upon during early discussion of constraints, expectations, and processes?</t>
+  </si>
+  <si>
+    <t>duration and frequency of team meetings</t>
+  </si>
+  <si>
+    <t>supplier selection criteria</t>
+  </si>
+  <si>
+    <t>terms and conditions for paid leave policy</t>
+  </si>
+  <si>
+    <t>pay rates for contractors</t>
+  </si>
+  <si>
+    <t>Exam questions</t>
+  </si>
+  <si>
+    <t>Filter results by</t>
+  </si>
+  <si>
+    <t>Show all</t>
+  </si>
+  <si>
+    <t>Show wrong only</t>
+  </si>
+  <si>
+    <t>Question 1 of 7</t>
+  </si>
+  <si>
+    <t>Attempted incorrect option</t>
+  </si>
+  <si>
+    <t>Correct answer</t>
+  </si>
+  <si>
+    <t>Question 2 of 7</t>
+  </si>
+  <si>
+    <t>Question 3 of 7</t>
+  </si>
+  <si>
+    <t>Attempted correct option</t>
+  </si>
+  <si>
+    <t>Question 4 of 7</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The primary benefit of a debrief is to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.6"/>
+        <color theme="1"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>_____</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Question 5 of 7</t>
+  </si>
+  <si>
+    <t>Question 6 of 7</t>
+  </si>
+  <si>
+    <t>Question 7 of 7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF2F7B15"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFD11124"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.6"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -359,7 +779,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -367,12 +787,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCDCFD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD11124"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD11124"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFD11124"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD11124"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF2F7B15"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF2F7B15"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF2F7B15"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF2F7B15"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,6 +893,119 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/activeX/activeX1.xml><?xml version="1.0" encoding="utf-8"?>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{5512D118-5CC6-11CF-8D67-00AA00BDCE1D}" ax:persistence="persistStream" r:id="rId1"/>
+</file>
+
+<file path=xl/activeX/activeX2.xml><?xml version="1.0" encoding="utf-8"?>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{5512D118-5CC6-11CF-8D67-00AA00BDCE1D}" ax:persistence="persistStream" r:id="rId1"/>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>94</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>257175</xdr:colOff>
+          <xdr:row>95</xdr:row>
+          <xdr:rowOff>76200</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1032" name="Control 8" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1032"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E11B16A5-2BB6-FFF9-1842-CB2513D4DDC3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>95</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>257175</xdr:colOff>
+          <xdr:row>96</xdr:row>
+          <xdr:rowOff>76200</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1033" name="Control 9" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1033"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54076EA7-FF29-4B6A-4246-63EF704EE9E2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1565,4 +2183,2402 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C94071-4E68-48D6-B9B0-2D652367C7D6}">
+  <sheetPr codeName="Sheet1" filterMode="1"/>
+  <dimension ref="A1:I198"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="5"/>
+    <col min="7" max="7" width="107" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="119.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="b">
+        <f>OR(NOT(ISERROR(FIND("m ",A4))),(RIGHT(A4,1)="m"))</f>
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <f>IF(C3&lt;&gt;C2,0,IF(B3,D2+1,D2))</f>
+        <v>0</v>
+      </c>
+      <c r="F3"/>
+    </row>
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" t="str">
+        <f>IF(ISERROR(FIND(". ",A4)),C3,A4)</f>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D59" si="0">IF(C4&lt;&gt;C3,0,IF(B4,D3+1,D3))</f>
+        <v>0</v>
+      </c>
+      <c r="E4" t="str">
+        <f>IF(B4,D4&amp;". "&amp;A4,"")</f>
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" ref="F4:F35" si="1">IF(B4,A5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" t="b">
+        <f>ISNUMBER(VALUE(LEFT(A6,FIND("m ",A6)-1)))</f>
+        <v>1</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" ref="C5:C59" si="2">IF(ISERROR(FIND(". ",A5)),C4,A5)</f>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" ref="E5:E59" si="3">IF(B5,D5&amp;". "&amp;A5,"")</f>
+        <v>1. Welcome to Essentials of Team Collaboration</v>
+      </c>
+      <c r="F5" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>1m 38s</v>
+      </c>
+      <c r="G5" t="str">
+        <f>IF(B5,C5&amp;" ("&amp;E5&amp;")","")</f>
+        <v>0. Introduction (1. Welcome to Essentials of Team Collaboration)</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="b">
+        <f t="shared" ref="B6:B59" si="4">ISNUMBER(VALUE(LEFT(A7,FIND("m ",A7)-1)))</f>
+        <v>0</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="2"/>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" ref="G6:G59" si="5">IF(B6,C6&amp;" ("&amp;E6&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="2"/>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="3"/>
+        <v>2. Why team collaboration is necessary</v>
+      </c>
+      <c r="F7" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>3m 27s</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="5"/>
+        <v>0. Introduction (2. Why team collaboration is necessary)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="2"/>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="2"/>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B10" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="2"/>
+        <v>0. Introduction</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="3"/>
+        <v>1. Six key questions for effective collaboration</v>
+      </c>
+      <c r="F13" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>2m 51s</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="5"/>
+        <v>1. Setting the Stage for Strong Team Collaboration (1. Six key questions for effective collaboration)</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="3"/>
+        <v>2. Identify the right team composition</v>
+      </c>
+      <c r="F16" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>2m 22s</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="5"/>
+        <v>1. Setting the Stage for Strong Team Collaboration (2. Identify the right team composition)</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="3"/>
+        <v>3. Clarify the team's goal and purpose</v>
+      </c>
+      <c r="F19" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>2m 37s</v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="5"/>
+        <v>1. Setting the Stage for Strong Team Collaboration (3. Clarify the team's goal and purpose)</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="3"/>
+        <v>4. Clarify constraints, expectations, and processes up front</v>
+      </c>
+      <c r="F22" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>2m 24s</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="5"/>
+        <v>1. Setting the Stage for Strong Team Collaboration (4. Clarify constraints, expectations, and processes up front)</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B27" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="2"/>
+        <v>1. Setting the Stage for Strong Team Collaboration</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B29" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="3"/>
+        <v>1. Develop team ground rules</v>
+      </c>
+      <c r="F30" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>2m 16s</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (1. Develop team ground rules)</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>116</v>
+      </c>
+      <c r="B31" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="3"/>
+        <v>2. Build relationships early and often(Viewed)</v>
+      </c>
+      <c r="F33" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>3m 7s</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (2. Build relationships early and often(Viewed))</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B35" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D35">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="3"/>
+        <v>3. Identify team members' preferred communication mode</v>
+      </c>
+      <c r="F36" s="5" t="str">
+        <f t="shared" ref="F36:F59" si="6">IF(B36,A37,"")</f>
+        <v>2m 39s</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (3. Identify team members' preferred communication mode)</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B39" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="3"/>
+        <v>4. Tips for great online collaboration</v>
+      </c>
+      <c r="F39" s="5" t="str">
+        <f t="shared" si="6"/>
+        <v>2m 56s</v>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (4. Tips for great online collaboration)</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>122</v>
+      </c>
+      <c r="B40" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E40" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E41" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E42" t="str">
+        <f t="shared" si="3"/>
+        <v>5. Take periodic temperature checks</v>
+      </c>
+      <c r="F42" s="5" t="str">
+        <f t="shared" si="6"/>
+        <v>2m 23s</v>
+      </c>
+      <c r="G42" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (5. Take periodic temperature checks)</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>124</v>
+      </c>
+      <c r="B43" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D43">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E43" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D44">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E44" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E45" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E46" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B47" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E47" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>126</v>
+      </c>
+      <c r="B48" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E48" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B49" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D49">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E49" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D50">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="3"/>
+        <v>6. Develop best practices to enhance team collaboration</v>
+      </c>
+      <c r="F50" s="5" t="str">
+        <f t="shared" si="6"/>
+        <v>2m 24s</v>
+      </c>
+      <c r="G50" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (6. Develop best practices to enhance team collaboration)</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B51" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C51" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D51">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E51" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C52" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D52">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E52" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="C53" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D53">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E53" t="str">
+        <f t="shared" si="3"/>
+        <v>7. Team collaboration challenge</v>
+      </c>
+      <c r="F53" s="5" t="str">
+        <f t="shared" si="6"/>
+        <v>1m 31s</v>
+      </c>
+      <c r="G53" t="str">
+        <f t="shared" si="5"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration (7. Team collaboration challenge)</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>129</v>
+      </c>
+      <c r="B54" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D54">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E54" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>102</v>
+      </c>
+      <c r="B55" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D55">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E55" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D56">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E56" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>130</v>
+      </c>
+      <c r="B57" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E57" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B58" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E58" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>131</v>
+      </c>
+      <c r="B59" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="2"/>
+        <v>2. Five Tactics to Encourage Healthy Team Collaboration</v>
+      </c>
+      <c r="D59">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E59" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F66" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="67" spans="6:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="G67" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="68" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F68" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69" spans="6:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="G69" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="70" spans="6:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F70" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="6:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="G71" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="72" spans="6:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F72" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="G72" s="4"/>
+    </row>
+    <row r="73" spans="6:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="G73" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="75" spans="6:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F75" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G75" s="6"/>
+    </row>
+    <row r="76" spans="6:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="G76" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F77" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="G77" s="4"/>
+    </row>
+    <row r="78" spans="6:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="G78" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="79" spans="6:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F79" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G79" s="4"/>
+    </row>
+    <row r="80" spans="6:7" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G80" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="81" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F81" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="82" spans="6:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="G82" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="83" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F83" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="84" spans="6:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="G84" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="85" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F85" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="86" spans="6:9" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G86" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="87" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F87" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="88" spans="6:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="G88" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="89" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F89" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="90" spans="6:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="G90" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="93" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I93" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="94" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F94" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="I94" s="12" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="95" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G95" s="7"/>
+      <c r="I95" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="96" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G96" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I96" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="97" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G97" s="9"/>
+      <c r="I97" s="7"/>
+    </row>
+    <row r="98" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G98" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="I98" s="13" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="99" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G99" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="I99" s="7"/>
+    </row>
+    <row r="100" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G100" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="I100" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="101" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G101" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="I101" s="14"/>
+    </row>
+    <row r="102" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I102" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="103" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F103" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I103" s="14"/>
+    </row>
+    <row r="104" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G104" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I104" s="8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="105" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G105" s="9"/>
+      <c r="I105" s="7"/>
+    </row>
+    <row r="106" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G106" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I106" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="107" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G107" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="I107" s="15"/>
+    </row>
+    <row r="108" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G108" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="I108" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="109" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G109" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="I109" s="15"/>
+    </row>
+    <row r="110" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I110" s="8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="111" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F111" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="I111" s="7"/>
+    </row>
+    <row r="112" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G112" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I112" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="113" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G113" s="9"/>
+      <c r="I113" s="7"/>
+    </row>
+    <row r="114" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G114" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="I114" s="13" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="115" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G115" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="I115" s="7"/>
+    </row>
+    <row r="116" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G116" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="I116" s="8" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="117" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G117" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="I117" s="14"/>
+    </row>
+    <row r="118" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F118" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="I118" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="119" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G119" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I119" s="14"/>
+    </row>
+    <row r="120" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G120" s="9"/>
+      <c r="I120" s="8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="121" spans="6:9" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G121" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="I121" s="15"/>
+    </row>
+    <row r="122" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G122" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="I122" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="123" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G123" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="I123" s="15"/>
+    </row>
+    <row r="124" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G124" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="I124" s="8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="125" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="I125" s="7"/>
+    </row>
+    <row r="126" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="F126" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="I126" s="8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="127" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G127" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I127" s="7"/>
+    </row>
+    <row r="128" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G128" s="9"/>
+      <c r="I128" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="129" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G129" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="I129" s="7"/>
+    </row>
+    <row r="130" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G130" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="I130" s="16" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="131" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G131" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="I131" s="7"/>
+    </row>
+    <row r="132" spans="6:9" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="G132" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="I132" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="133" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="I133" s="7"/>
+    </row>
+    <row r="134" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F134" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="I134" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="135" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G135" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I135" s="15"/>
+    </row>
+    <row r="136" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G136" s="9"/>
+      <c r="I136" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="137" spans="6:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G137" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="I137" s="15"/>
+    </row>
+    <row r="138" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G138" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="I138" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="139" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G139" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="I139" s="7"/>
+    </row>
+    <row r="140" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G140" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="I140" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="141" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="I141" s="7"/>
+    </row>
+    <row r="142" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="F142" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="I142" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="143" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G143" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I143" s="7"/>
+    </row>
+    <row r="144" spans="6:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G144" s="9"/>
+      <c r="I144" s="16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="145" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="G145" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="I145" s="7"/>
+    </row>
+    <row r="146" spans="7:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G146" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="I146" s="8" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="147" spans="7:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G147" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="I147" s="15"/>
+    </row>
+    <row r="148" spans="7:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G148" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="I148" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="149" spans="7:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I149" s="15"/>
+    </row>
+    <row r="150" spans="7:9" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="I150" s="8" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="151" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I151" s="7"/>
+    </row>
+    <row r="152" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I152" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="153" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I153" s="7"/>
+    </row>
+    <row r="154" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I154" s="8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="155" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I155" s="7"/>
+    </row>
+    <row r="156" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I156" s="8" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="157" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I157" s="7"/>
+    </row>
+    <row r="158" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I158" s="16" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="159" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I159" s="7"/>
+    </row>
+    <row r="160" spans="7:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I160" s="8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="161" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I161" s="7"/>
+    </row>
+    <row r="162" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I162" s="8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="163" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I163" s="7"/>
+    </row>
+    <row r="164" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I164" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="165" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I165" s="7"/>
+    </row>
+    <row r="166" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I166" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="167" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I167" s="15"/>
+    </row>
+    <row r="168" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I168" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="169" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I169" s="15"/>
+    </row>
+    <row r="170" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I170" s="8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="171" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I171" s="7"/>
+    </row>
+    <row r="172" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I172" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="173" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I173" s="7"/>
+    </row>
+    <row r="174" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I174" s="8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="175" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I175" s="15"/>
+    </row>
+    <row r="176" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I176" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="177" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I177" s="15"/>
+    </row>
+    <row r="178" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I178" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="179" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I179" s="7"/>
+    </row>
+    <row r="180" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I180" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="181" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I181" s="7"/>
+    </row>
+    <row r="182" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I182" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="183" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I183" s="7"/>
+    </row>
+    <row r="184" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I184" s="8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="185" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I185" s="7"/>
+    </row>
+    <row r="186" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I186" s="16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="187" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I187" s="7"/>
+    </row>
+    <row r="188" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I188" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="189" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I189" s="15"/>
+    </row>
+    <row r="190" spans="9:9" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I190" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="191" spans="9:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I191" s="15"/>
+    </row>
+    <row r="192" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I192" s="8" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="193" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I193" s="7"/>
+    </row>
+    <row r="194" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I194" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="195" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I195" s="7"/>
+    </row>
+    <row r="196" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I196" s="8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="197" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I197" s="7"/>
+    </row>
+    <row r="198" spans="9:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="I198" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:G59" xr:uid="{39C94071-4E68-48D6-B9B0-2D652367C7D6}">
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
+  <mergeCells count="5">
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F79:G79"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <controls>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="1033" r:id="rId4" name="Control 9">
+          <controlPr defaultSize="0" r:id="rId5">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>95</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>257175</xdr:colOff>
+                <xdr:row>96</xdr:row>
+                <xdr:rowOff>76200</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="1033" r:id="rId4" name="Control 9"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="1032" r:id="rId6" name="Control 8">
+          <controlPr defaultSize="0" r:id="rId5">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>94</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>257175</xdr:colOff>
+                <xdr:row>95</xdr:row>
+                <xdr:rowOff>76200</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="1032" r:id="rId6" name="Control 8"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </controls>
+</worksheet>
 </file>
</xml_diff>